<commit_message>
Add water quality data
</commit_message>
<xml_diff>
--- a/08_sampledata.xlsx
+++ b/08_sampledata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/65f33c3464bcf092/Research/2018-2022_Sado/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="335" documentId="8_{C96D46A6-B296-FB4D-A5F1-3DE4A23156A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71A64F87-3ED3-514B-8C07-460D991ADC10}"/>
+  <xr:revisionPtr revIDLastSave="336" documentId="8_{C96D46A6-B296-FB4D-A5F1-3DE4A23156A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81ED2751-6676-CC46-91BB-99B45ABCFA29}"/>
   <bookViews>
     <workbookView xWindow="7940" yWindow="600" windowWidth="27160" windowHeight="27760" xr2:uid="{3521B622-29B9-CA4D-8B15-F4EE5C51B8FD}"/>
   </bookViews>
@@ -2898,10 +2898,6 @@
     <phoneticPr fontId="18"/>
   </si>
   <si>
-    <t>disch</t>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
     <t>sample</t>
     <phoneticPr fontId="18"/>
   </si>
@@ -2911,6 +2907,10 @@
   </si>
   <si>
     <t>ec</t>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>disc</t>
     <phoneticPr fontId="18"/>
   </si>
 </sst>
@@ -2919,9 +2919,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="179" formatCode="0.00_ "/>
-    <numFmt numFmtId="180" formatCode="0.00_);[Red]\(0.00\)"/>
-    <numFmt numFmtId="182" formatCode="0.0_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
+    <numFmt numFmtId="177" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="178" formatCode="0.0_ "/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -3519,13 +3519,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3931,7 +3931,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B1" t="s">
         <v>474</v>
@@ -3985,13 +3985,13 @@
         <v>925</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="T1" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="U1" t="s">
         <v>928</v>
-      </c>
-      <c r="U1" t="s">
-        <v>929</v>
       </c>
     </row>
     <row r="2" spans="1:21">

</xml_diff>